<commit_message>
Change zero-dollar sentinel from 0.000001 to 0.0001
Downstream ingestion was rejecting the previous sentinel. Centralised the
value as TemplateLayout.ZeroPriceSentinel so all four output templates
(Foreign Uplift, No Calculation, Uplift, % Off RRP with Uplift) share one
source of truth. Regenerated golden fixtures, updated tests, comments, and
AGENTS.md.
</commit_message>
<xml_diff>
--- a/samples/outputs/55648855_parsed.xlsx
+++ b/samples/outputs/55648855_parsed.xlsx
@@ -876,7 +876,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K4" s="0">
         <x:v>5</x:v>
@@ -902,7 +902,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K5" s="0">
         <x:v>5</x:v>
@@ -928,7 +928,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K6" s="0">
         <x:v>5</x:v>
@@ -954,7 +954,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K7" s="0">
         <x:v>5</x:v>
@@ -980,7 +980,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K8" s="0">
         <x:v>5</x:v>
@@ -1006,7 +1006,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K9" s="0">
         <x:v>5</x:v>
@@ -1032,7 +1032,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H10" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K10" s="0">
         <x:v>5</x:v>
@@ -1058,7 +1058,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K11" s="0">
         <x:v>5</x:v>
@@ -1084,7 +1084,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K12" s="0">
         <x:v>5</x:v>
@@ -1110,7 +1110,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K13" s="0">
         <x:v>5</x:v>
@@ -1136,7 +1136,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K14" s="0">
         <x:v>5</x:v>
@@ -1162,7 +1162,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K15" s="0">
         <x:v>5</x:v>
@@ -1188,7 +1188,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K16" s="0">
         <x:v>5</x:v>
@@ -1214,7 +1214,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K17" s="0">
         <x:v>5</x:v>
@@ -1240,7 +1240,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K18" s="0">
         <x:v>5</x:v>
@@ -1266,7 +1266,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K19" s="0">
         <x:v>5</x:v>
@@ -1292,7 +1292,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K20" s="0">
         <x:v>5</x:v>
@@ -1318,7 +1318,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K21" s="0">
         <x:v>5</x:v>
@@ -1344,7 +1344,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K22" s="0">
         <x:v>5</x:v>
@@ -1370,7 +1370,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K23" s="0">
         <x:v>5</x:v>
@@ -1396,7 +1396,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K24" s="0">
         <x:v>5</x:v>
@@ -1422,7 +1422,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K25" s="0">
         <x:v>5</x:v>
@@ -1448,7 +1448,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K26" s="0">
         <x:v>5</x:v>
@@ -1474,7 +1474,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K27" s="0">
         <x:v>5</x:v>
@@ -1500,7 +1500,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K28" s="0">
         <x:v>5</x:v>
@@ -1526,7 +1526,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H29" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K29" s="0">
         <x:v>5</x:v>
@@ -1552,7 +1552,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H30" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K30" s="0">
         <x:v>5</x:v>
@@ -1578,7 +1578,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H31" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K31" s="0">
         <x:v>5</x:v>
@@ -1604,7 +1604,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H32" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K32" s="0">
         <x:v>5</x:v>
@@ -1630,7 +1630,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H33" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>0.0001</x:v>
       </x:c>
       <x:c r="K33" s="0">
         <x:v>5</x:v>

</xml_diff>

<commit_message>
HP Bid + OneConfig (XLSX): flatten line numbering to a single 1..N sequence
Bundle Detail rows (HP Bid) and component rows (OneConfig) are no longer
sub-numbered under their parent (1.01, 1.02, ...); every emitted line now
takes the next number in one running sequence. Comment placement is
unchanged (Max Qty only on Part Number/Bundle lines). Updated parser tests,
regenerated the affected goldens, and refreshed the HP format specs +
output mapping docs.
</commit_message>
<xml_diff>
--- a/samples/outputs/55648855_parsed.xlsx
+++ b/samples/outputs/55648855_parsed.xlsx
@@ -114,7 +114,7 @@
     <x:t>HP EliteBook 6 G2i 14 AI</x:t>
   </x:si>
   <x:si>
-    <x:t>1.01</x:t>
+    <x:t>2</x:t>
   </x:si>
   <x:si>
     <x:t>C6SL9AV</x:t>
@@ -123,7 +123,7 @@
     <x:t>HP IDS UMA Ultra 7 355 for WWAN 6 14 inch G2i Base NB PC</x:t>
   </x:si>
   <x:si>
-    <x:t>1.02</x:t>
+    <x:t>3</x:t>
   </x:si>
   <x:si>
     <x:t>8C9M7AV</x:t>
@@ -132,7 +132,7 @@
     <x:t>No Country of Origin Restriction</x:t>
   </x:si>
   <x:si>
-    <x:t>1.03</x:t>
+    <x:t>4</x:t>
   </x:si>
   <x:si>
     <x:t>1Y629AV</x:t>
@@ -141,7 +141,7 @@
     <x:t>Electronic Energy Star labeling (EStar)</x:t>
   </x:si>
   <x:si>
-    <x:t>1.04</x:t>
+    <x:t>5</x:t>
   </x:si>
   <x:si>
     <x:t>C71WMAV</x:t>
@@ -150,7 +150,7 @@
     <x:t>Windows 11 Pro 64 NextGen Premium</x:t>
   </x:si>
   <x:si>
-    <x:t>1.05</x:t>
+    <x:t>6</x:t>
   </x:si>
   <x:si>
     <x:t>4SS11AV#ABG</x:t>
@@ -159,7 +159,7 @@
     <x:t>OS Localization AUST</x:t>
   </x:si>
   <x:si>
-    <x:t>1.06</x:t>
+    <x:t>7</x:t>
   </x:si>
   <x:si>
     <x:t>D0AN1AV</x:t>
@@ -168,7 +168,7 @@
     <x:t>Dual AryMic 5MP USB2 IR AI WFOV Integrated Camera</x:t>
   </x:si>
   <x:si>
-    <x:t>1.07</x:t>
+    <x:t>8</x:t>
   </x:si>
   <x:si>
     <x:t>C71VKAV</x:t>
@@ -177,7 +177,7 @@
     <x:t>14.0 inch AG WUXGA (1920x1200) LED UWVA 300 for WWAN f5MP IR ISP+ 60Hz bnt LCD Panel</x:t>
   </x:si>
   <x:si>
-    <x:t>1.08</x:t>
+    <x:t>9</x:t>
   </x:si>
   <x:si>
     <x:t>CK0F3AV</x:t>
@@ -186,7 +186,7 @@
     <x:t>32GB (1x32GB) DDR5 5600 SODIMM NMIC Memory</x:t>
   </x:si>
   <x:si>
-    <x:t>1.09</x:t>
+    <x:t>10</x:t>
   </x:si>
   <x:si>
     <x:t>CK0F8AV</x:t>
@@ -195,7 +195,7 @@
     <x:t>512GB PCIe Gen5 2280 NVMe Value NMIC Solid State Drive</x:t>
   </x:si>
   <x:si>
-    <x:t>1.10</x:t>
+    <x:t>11</x:t>
   </x:si>
   <x:si>
     <x:t>C71U9AV</x:t>
@@ -204,7 +204,7 @@
     <x:t>Pike Silver Aluminum for WWAN 20W ID</x:t>
   </x:si>
   <x:si>
-    <x:t>1.11</x:t>
+    <x:t>12</x:t>
   </x:si>
   <x:si>
     <x:t>C71W2AV</x:t>
@@ -213,7 +213,7 @@
     <x:t>WNC XRAV-1 NFC</x:t>
   </x:si>
   <x:si>
-    <x:t>1.12</x:t>
+    <x:t>13</x:t>
   </x:si>
   <x:si>
     <x:t>C71Y3AV</x:t>
@@ -222,7 +222,7 @@
     <x:t>Intel AX211 Wi-Fi 6E +Bluetooth 5.3 WW WLAN</x:t>
   </x:si>
   <x:si>
-    <x:t>1.13</x:t>
+    <x:t>14</x:t>
   </x:si>
   <x:si>
     <x:t>C71Y7AV</x:t>
@@ -231,7 +231,7 @@
     <x:t>MediaTek T700 5G NR/4G WWAN</x:t>
   </x:si>
   <x:si>
-    <x:t>1.14</x:t>
+    <x:t>15</x:t>
   </x:si>
   <x:si>
     <x:t>C71XCAV</x:t>
@@ -240,7 +240,7 @@
     <x:t>Fingerprint Sensor</x:t>
   </x:si>
   <x:si>
-    <x:t>1.15</x:t>
+    <x:t>16</x:t>
   </x:si>
   <x:si>
     <x:t>C71XBAV</x:t>
@@ -249,7 +249,7 @@
     <x:t>Active SmartCard</x:t>
   </x:si>
   <x:si>
-    <x:t>1.16</x:t>
+    <x:t>17</x:t>
   </x:si>
   <x:si>
     <x:t>C71U5AV</x:t>
@@ -258,7 +258,7 @@
     <x:t>PM Long Life 68Whr Fast Charge 3 cell Battery</x:t>
   </x:si>
   <x:si>
-    <x:t>1.17</x:t>
+    <x:t>18</x:t>
   </x:si>
   <x:si>
     <x:t>C71TWAV</x:t>
@@ -267,7 +267,7 @@
     <x:t>HP 100W Gallium Nitride Wmnt USB-C Halogen Free Fixed AC Adapter</x:t>
   </x:si>
   <x:si>
-    <x:t>1.18</x:t>
+    <x:t>19</x:t>
   </x:si>
   <x:si>
     <x:t>C72MSAV#ABG</x:t>
@@ -276,7 +276,7 @@
     <x:t>for TBT Clickpad for NFC Backlit spill-resistant KBD</x:t>
   </x:si>
   <x:si>
-    <x:t>1.19</x:t>
+    <x:t>20</x:t>
   </x:si>
   <x:si>
     <x:t>C72MNAV#ABG</x:t>
@@ -285,7 +285,7 @@
     <x:t>Country Localization</x:t>
   </x:si>
   <x:si>
-    <x:t>1.20</x:t>
+    <x:t>21</x:t>
   </x:si>
   <x:si>
     <x:t>D4JJ8AV#ABG</x:t>
@@ -294,7 +294,7 @@
     <x:t>Non-Standard Straight Halogen Free Non-China Duckhead Only</x:t>
   </x:si>
   <x:si>
-    <x:t>1.21</x:t>
+    <x:t>22</x:t>
   </x:si>
   <x:si>
     <x:t>C72MPAV#UUF</x:t>
@@ -303,7 +303,7 @@
     <x:t>1/1/1 Warranty</x:t>
   </x:si>
   <x:si>
-    <x:t>1.22</x:t>
+    <x:t>23</x:t>
   </x:si>
   <x:si>
     <x:t>791T2AV</x:t>
@@ -312,7 +312,7 @@
     <x:t>Pre-Boot UEFI Wi-Fi support</x:t>
   </x:si>
   <x:si>
-    <x:t>1.23</x:t>
+    <x:t>24</x:t>
   </x:si>
   <x:si>
     <x:t>4N735AV</x:t>
@@ -321,7 +321,7 @@
     <x:t>HP Tamper Lock</x:t>
   </x:si>
   <x:si>
-    <x:t>1.24</x:t>
+    <x:t>25</x:t>
   </x:si>
   <x:si>
     <x:t>X9H42AV</x:t>
@@ -330,7 +330,7 @@
     <x:t>No vPro AMT supported</x:t>
   </x:si>
   <x:si>
-    <x:t>1.25</x:t>
+    <x:t>26</x:t>
   </x:si>
   <x:si>
     <x:t>C71W1AV</x:t>
@@ -339,7 +339,7 @@
     <x:t>Standard Packaging</x:t>
   </x:si>
   <x:si>
-    <x:t>1.26</x:t>
+    <x:t>27</x:t>
   </x:si>
   <x:si>
     <x:t>D18SMAV</x:t>
@@ -348,7 +348,7 @@
     <x:t>HP Sure Recover Enhanced Local Storage Disable - Gen5 drive required</x:t>
   </x:si>
   <x:si>
-    <x:t>1.27</x:t>
+    <x:t>28</x:t>
   </x:si>
   <x:si>
     <x:t>3E755AV</x:t>
@@ -357,7 +357,7 @@
     <x:t>Electronic TCO Certified labeling</x:t>
   </x:si>
   <x:si>
-    <x:t>1.28</x:t>
+    <x:t>29</x:t>
   </x:si>
   <x:si>
     <x:t>C1GT2AV</x:t>
@@ -366,7 +366,7 @@
     <x:t>Intel Core Ultra 7 sz3 G18 Label</x:t>
   </x:si>
   <x:si>
-    <x:t>1.29</x:t>
+    <x:t>30</x:t>
   </x:si>
   <x:si>
     <x:t>X7A78AV</x:t>
@@ -375,7 +375,7 @@
     <x:t>Warranty Book 2016 AP 1YR</x:t>
   </x:si>
   <x:si>
-    <x:t>1.30</x:t>
+    <x:t>31</x:t>
   </x:si>
   <x:si>
     <x:t>U85GJE</x:t>

</xml_diff>